<commit_message>
Temperature, Time-range and field pig
Changed temperature to 20 cm above ground for field cattle

Changed algorithm to determine common time-range, as the former "falied" when applied to pig slurry

Produced accumulated emissions for pig slurry
</commit_message>
<xml_diff>
--- a/Field-trails/TAN-concentration-and-aplication-rate.xlsx
+++ b/Field-trails/TAN-concentration-and-aplication-rate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Field-trails\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F58DC15-0D47-444C-9511-C6708A8D6D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7992FA78-A176-4CFB-94E5-3E0FE14AB35C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -583,7 +583,7 @@
         <v>1.9151419999999999</v>
       </c>
       <c r="G3">
-        <f t="shared" ref="G3:G22" si="1">E3*F3*10^3</f>
+        <f>E3*F3*10^3</f>
         <v>5553.9118000000008</v>
       </c>
     </row>
@@ -608,7 +608,7 @@
         <v>1.794495</v>
       </c>
       <c r="G4">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="G3:G22" si="1">E4*F4*10^3</f>
         <v>5204.0355000000009</v>
       </c>
       <c r="H4" s="2">

</xml_diff>

<commit_message>
Long time since update
Major changes
-started working with ALFAM2, changed folder-structure to better accomodate this

- Setup files for density test data treatment
</commit_message>
<xml_diff>
--- a/Field-trails/TAN-concentration-and-aplication-rate.xlsx
+++ b/Field-trails/TAN-concentration-and-aplication-rate.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Field-trails\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67F821B7-0800-4FD5-A76B-1308645F7679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4246A580-80A5-4593-99BD-0610B15522EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="18">
   <si>
     <t>Trial</t>
   </si>
@@ -126,6 +126,12 @@
   </si>
   <si>
     <t>AmmoniumN application rate mean [mg/m2]</t>
+  </si>
+  <si>
+    <t>AmmoniumN application rate [kg/ ha]</t>
+  </si>
+  <si>
+    <t>mean</t>
   </si>
 </sst>
 </file>
@@ -470,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
@@ -480,7 +486,7 @@
     <col min="6" max="9" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="72" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -508,12 +514,14 @@
       <c r="I1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K1" t="s">
+      <c r="J1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" t="s">
         <v>13</v>
       </c>
-      <c r="L1" s="1"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -537,8 +545,19 @@
         <f>E2*F2*10^3</f>
         <v>6316.5537275000006</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L2">
+        <f>AVERAGE(G2:G10)</f>
+        <v>6225.7384030777785</v>
+      </c>
+      <c r="M2" s="2">
+        <f>L2/100</f>
+        <v>62.257384030777786</v>
+      </c>
+      <c r="N2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -562,8 +581,16 @@
         <f>E3*F3*10^3</f>
         <v>6158.3011596000015</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L3">
+        <f>_xlfn.STDEV.P(G2:G10)</f>
+        <v>134.82711051118892</v>
+      </c>
+      <c r="M3" s="2">
+        <f>L3/100</f>
+        <v>1.3482711051118892</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -595,8 +622,12 @@
         <f>_xlfn.STDEV.P(G2:G4)</f>
         <v>119.19894847353086</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="J4">
+        <f>H4*10^-6*10^4</f>
+        <v>61.665952118000007</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -621,7 +652,7 @@
         <v>6001.8814671000009</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -645,12 +676,8 @@
         <f t="shared" si="1"/>
         <v>6397.0588237000002</v>
       </c>
-      <c r="K6">
-        <f>AVERAGE(G2:G22)</f>
-        <v>6211.6052419047619</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -682,8 +709,12 @@
         <f>_xlfn.STDEV.P(G5:G7)</f>
         <v>181.01826145254597</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="J7">
+        <f>H7/100</f>
+        <v>62.575222216666674</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -708,7 +739,7 @@
         <v>6185.5158732</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -733,7 +764,7 @@
         <v>6292.189006300001</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -765,8 +796,12 @@
         <f>_xlfn.STDEV.P(G8:G10)</f>
         <v>47.983178483199438</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="J10">
+        <f>H10/100</f>
+        <v>62.530977757666669</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -791,7 +826,7 @@
         <v>6133.2099911000014</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -816,7 +851,7 @@
         <v>6041.4610064000008</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>6</v>
       </c>
@@ -848,8 +883,12 @@
         <f>_xlfn.STDEV.P(G11:G13)</f>
         <v>203.03183484844897</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="J13">
+        <f>H13/100</f>
+        <v>62.284364317666672</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -874,7 +913,7 @@
         <v>6245.7770262000004</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>6</v>
       </c>
@@ -899,7 +938,7 @@
         <v>6326.3358782000014</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>6</v>
       </c>
@@ -931,8 +970,12 @@
         <f>_xlfn.STDEV.P(G14:G16)</f>
         <v>62.014021128701707</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J16">
+        <f>H16/100</f>
+        <v>62.48880402266667</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>6</v>
       </c>
@@ -957,7 +1000,7 @@
         <v>6145.6211811000003</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>6</v>
       </c>
@@ -982,7 +1025,7 @@
         <v>6236.1809053000006</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>6</v>
       </c>
@@ -1014,8 +1057,12 @@
         <f>_xlfn.STDEV.P(G17:G19)</f>
         <v>113.80078787884609</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J19">
+        <f>H19/100</f>
+        <v>61.147965907000007</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>6</v>
       </c>
@@ -1040,7 +1087,7 @@
         <v>6277.9397478000001</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>6</v>
       </c>
@@ -1065,7 +1112,7 @@
         <v>6249.9999996000006</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>6</v>
       </c>
@@ -1096,6 +1143,10 @@
       <c r="I22" s="2">
         <f>_xlfn.STDEV.P(G20:G22)</f>
         <v>74.504831688534338</v>
+      </c>
+      <c r="J22">
+        <f>H22/100</f>
+        <v>62.119080593666666</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
weather-data for alfram modelling
created a new csv-file for ALfAM modelling
</commit_message>
<xml_diff>
--- a/Field-trails/TAN-concentration-and-aplication-rate.xlsx
+++ b/Field-trails/TAN-concentration-and-aplication-rate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Field-trails\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4246A580-80A5-4593-99BD-0610B15522EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D7B65D7-F957-4435-A5F0-50D3188F9868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="20">
   <si>
     <t>Trial</t>
   </si>
@@ -132,6 +132,12 @@
   </si>
   <si>
     <t>mean</t>
+  </si>
+  <si>
+    <t>AmmoniumN application rate stdev [kg/ha]</t>
+  </si>
+  <si>
+    <t>=</t>
   </si>
 </sst>
 </file>
@@ -476,7 +482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
@@ -486,7 +492,7 @@
     <col min="6" max="9" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -517,11 +523,14 @@
       <c r="J1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="L1" t="s">
+      <c r="K1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="M1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -545,19 +554,19 @@
         <f>E2*F2*10^3</f>
         <v>6316.5537275000006</v>
       </c>
-      <c r="L2">
+      <c r="M2">
         <f>AVERAGE(G2:G10)</f>
         <v>6225.7384030777785</v>
       </c>
-      <c r="M2" s="2">
-        <f>L2/100</f>
+      <c r="N2" s="2">
+        <f>M2/100</f>
         <v>62.257384030777786</v>
       </c>
-      <c r="N2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -581,16 +590,16 @@
         <f>E3*F3*10^3</f>
         <v>6158.3011596000015</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <f>_xlfn.STDEV.P(G2:G10)</f>
         <v>134.82711051118892</v>
       </c>
-      <c r="M3" s="2">
-        <f>L3/100</f>
+      <c r="N3" s="2">
+        <f>M3/100</f>
         <v>1.3482711051118892</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -626,8 +635,12 @@
         <f>H4*10^-6*10^4</f>
         <v>61.665952118000007</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="K4">
+        <f>I4/100</f>
+        <v>1.1919894847353085</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -652,7 +665,7 @@
         <v>6001.8814671000009</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -677,7 +690,7 @@
         <v>6397.0588237000002</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -713,8 +726,12 @@
         <f>H7/100</f>
         <v>62.575222216666674</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="K7">
+        <f>I7/100</f>
+        <v>1.8101826145254598</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -739,7 +756,7 @@
         <v>6185.5158732</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -764,7 +781,7 @@
         <v>6292.189006300001</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -800,8 +817,12 @@
         <f>H10/100</f>
         <v>62.530977757666669</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="K10">
+        <f>I10/100</f>
+        <v>0.4798317848319944</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -826,7 +847,7 @@
         <v>6133.2099911000014</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -851,7 +872,7 @@
         <v>6041.4610064000008</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>6</v>
       </c>
@@ -887,8 +908,12 @@
         <f>H13/100</f>
         <v>62.284364317666672</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="K13">
+        <f>I13/100</f>
+        <v>2.0303183484844896</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -913,7 +938,7 @@
         <v>6245.7770262000004</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>6</v>
       </c>
@@ -938,7 +963,7 @@
         <v>6326.3358782000014</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>6</v>
       </c>
@@ -974,8 +999,12 @@
         <f>H16/100</f>
         <v>62.48880402266667</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K16">
+        <f>H16/100</f>
+        <v>62.48880402266667</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>6</v>
       </c>
@@ -1000,7 +1029,7 @@
         <v>6145.6211811000003</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>6</v>
       </c>
@@ -1025,7 +1054,7 @@
         <v>6236.1809053000006</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>6</v>
       </c>
@@ -1061,8 +1090,11 @@
         <f>H19/100</f>
         <v>61.147965907000007</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K19" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>6</v>
       </c>
@@ -1087,7 +1119,7 @@
         <v>6277.9397478000001</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>6</v>
       </c>
@@ -1112,7 +1144,7 @@
         <v>6249.9999996000006</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
Completed data treatment of Density-test
</commit_message>
<xml_diff>
--- a/Field-trails/TAN-concentration-and-aplication-rate.xlsx
+++ b/Field-trails/TAN-concentration-and-aplication-rate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Field-trails\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D7B65D7-F957-4435-A5F0-50D3188F9868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48D4C974-E71C-4238-8B2E-E7682C274351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="19">
   <si>
     <t>Trial</t>
   </si>
@@ -136,14 +136,14 @@
   <si>
     <t>AmmoniumN application rate stdev [kg/ha]</t>
   </si>
-  <si>
-    <t>=</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="0.0"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -181,12 +181,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -490,6 +491,7 @@
     <col min="4" max="4" width="13.33203125" customWidth="1"/>
     <col min="5" max="5" width="13.33203125" style="1" customWidth="1"/>
     <col min="6" max="9" width="13.33203125" customWidth="1"/>
+    <col min="10" max="11" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
@@ -631,11 +633,11 @@
         <f>_xlfn.STDEV.P(G2:G4)</f>
         <v>119.19894847353086</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="2">
         <f>H4*10^-6*10^4</f>
         <v>61.665952118000007</v>
       </c>
-      <c r="K4">
+      <c r="K4" s="2">
         <f>I4/100</f>
         <v>1.1919894847353085</v>
       </c>
@@ -722,11 +724,11 @@
         <f>_xlfn.STDEV.P(G5:G7)</f>
         <v>181.01826145254597</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="2">
         <f>H7/100</f>
         <v>62.575222216666674</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="2">
         <f>I7/100</f>
         <v>1.8101826145254598</v>
       </c>
@@ -813,11 +815,11 @@
         <f>_xlfn.STDEV.P(G8:G10)</f>
         <v>47.983178483199438</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="3">
         <f>H10/100</f>
         <v>62.530977757666669</v>
       </c>
-      <c r="K10">
+      <c r="K10" s="3">
         <f>I10/100</f>
         <v>0.4798317848319944</v>
       </c>
@@ -904,14 +906,8 @@
         <f>_xlfn.STDEV.P(G11:G13)</f>
         <v>203.03183484844897</v>
       </c>
-      <c r="J13">
-        <f>H13/100</f>
-        <v>62.284364317666672</v>
-      </c>
-      <c r="K13">
-        <f>I13/100</f>
-        <v>2.0303183484844896</v>
-      </c>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -995,16 +991,8 @@
         <f>_xlfn.STDEV.P(G14:G16)</f>
         <v>62.014021128701707</v>
       </c>
-      <c r="J16">
-        <f>H16/100</f>
-        <v>62.48880402266667</v>
-      </c>
-      <c r="K16">
-        <f>H16/100</f>
-        <v>62.48880402266667</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>6</v>
       </c>
@@ -1029,7 +1017,7 @@
         <v>6145.6211811000003</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>6</v>
       </c>
@@ -1054,7 +1042,7 @@
         <v>6236.1809053000006</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>6</v>
       </c>
@@ -1086,15 +1074,8 @@
         <f>_xlfn.STDEV.P(G17:G19)</f>
         <v>113.80078787884609</v>
       </c>
-      <c r="J19">
-        <f>H19/100</f>
-        <v>61.147965907000007</v>
-      </c>
-      <c r="K19" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>6</v>
       </c>
@@ -1119,7 +1100,7 @@
         <v>6277.9397478000001</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>6</v>
       </c>
@@ -1144,7 +1125,7 @@
         <v>6249.9999996000006</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>6</v>
       </c>
@@ -1175,10 +1156,6 @@
       <c r="I22" s="2">
         <f>_xlfn.STDEV.P(G20:G22)</f>
         <v>74.504831688534338</v>
-      </c>
-      <c r="J22">
-        <f>H22/100</f>
-        <v>62.119080593666666</v>
       </c>
     </row>
   </sheetData>

</xml_diff>